<commit_message>
#7 Changes in Control Board completed
</commit_message>
<xml_diff>
--- a/Design-Files-v2.5/Control-Board_v2.5/Deliverables/BOM/Control-Board_v2.5.xlsx
+++ b/Design-Files-v2.5/Control-Board_v2.5/Deliverables/BOM/Control-Board_v2.5.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20415"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20416"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eSpark Cons Group\Documents\GitHub\Melih-SoundSensor\bradfairman-ledproject\Design-Files-v2.4\Control-Board_v2.4\Project Outputs for Control-Board_v2.4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eSpark Cons Group\Documents\GitHub\Melih-SoundSensor\bradfairman-ledproject\Design-Files-v2.5\Control-Board_v2.5\Project Outputs for Control-Board_v2.5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6234415-B42F-4E55-B028-4539071276CF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DFE20F3-885B-4FDA-B798-82AA13662B61}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="181">
   <si>
     <t>#</t>
   </si>
@@ -31,9 +31,6 @@
     <t>Capacitor</t>
   </si>
   <si>
-    <t>Capacitor, [NoParam]</t>
-  </si>
-  <si>
     <t>Diode</t>
   </si>
   <si>
@@ -70,10 +67,10 @@
     <t>Designator</t>
   </si>
   <si>
-    <t>C1</t>
-  </si>
-  <si>
-    <t>C2</t>
+    <t>C1, C10, C12</t>
+  </si>
+  <si>
+    <t>C2, C15</t>
   </si>
   <si>
     <t>C3, C7</t>
@@ -82,15 +79,9 @@
     <t>C4, C6, C8, C9</t>
   </si>
   <si>
-    <t>C10, C12</t>
-  </si>
-  <si>
     <t>C13, C14</t>
   </si>
   <si>
-    <t>C15</t>
-  </si>
-  <si>
     <t>D1</t>
   </si>
   <si>
@@ -124,7 +115,7 @@
     <t>Q6</t>
   </si>
   <si>
-    <t>R1, R2, R13</t>
+    <t>R1, R2, R5, R7, R9, R12, R13, R17, R19, R20, R26, R28, R30</t>
   </si>
   <si>
     <t>R3, R11, R21</t>
@@ -133,9 +124,6 @@
     <t>R4, R22, R23</t>
   </si>
   <si>
-    <t>R5, R7, R9, R12, R17, R19, R20, R26, R28, R30</t>
-  </si>
-  <si>
     <t>R6</t>
   </si>
   <si>
@@ -184,10 +172,10 @@
     <t>Description</t>
   </si>
   <si>
-    <t>CAP CER 1UF 10V X5R 0201</t>
-  </si>
-  <si>
-    <t>CAP CER 0.1UF 10V X5R 0201</t>
+    <t>CAP CER 1UF 16V X5R 0402, CAP CER 1UF 25V X5R 0402</t>
+  </si>
+  <si>
+    <t>CAP CER 0.1UF 16V X7R 0402</t>
   </si>
   <si>
     <t>CAP CER 4.7UF 16V X5R 0402</t>
@@ -196,15 +184,9 @@
     <t>CAP CER 10UF 10V X5R 0402</t>
   </si>
   <si>
-    <t>CAP CER 1UF 16V X5R 0402, CAP CER 1UF 25V X5R 0402</t>
-  </si>
-  <si>
     <t>CAP CER 0.68UF 10V X5R 0402</t>
   </si>
   <si>
-    <t>CAP CER 0.1UF 16V X7R 0402</t>
-  </si>
-  <si>
     <t>DIODE SCHOTTKY 40V 1A SOD123</t>
   </si>
   <si>
@@ -238,16 +220,13 @@
     <t>MOSFET N-CH 20V 630MA SOT523</t>
   </si>
   <si>
-    <t>RES SMD 10K OHM 1% 1/20W 0201</t>
+    <t>RES 10K OHM 1% 1/16W 0402, 10 kOhms ±1% 0.063W, 1/16W Chip Resistor 0402 (1005 Metric) Moisture Resistant Thick Film, RES SMD 10K OHM 0.1% 1/16W 0402</t>
   </si>
   <si>
     <t>RES SMD 1K OHM 1% 1/5W 0402, 1 kOhms ±1% 0.063W, 1/16W Chip Resistor 0402 (1005 Metric) Moisture Resistant Thick Film, RES 1K OHM 1% 1/16W 0402</t>
   </si>
   <si>
-    <t>RES 4.7K OHM 1% 1/20W 0201</t>
-  </si>
-  <si>
-    <t>RES 10K OHM 1% 1/16W 0402, 10 kOhms ±1% 0.063W, 1/16W Chip Resistor 0402 (1005 Metric) Moisture Resistant Thick Film, RES SMD 10K OHM 0.1% 1/16W 0402</t>
+    <t>RES 4.7K OHM 1% 1/16W 0402</t>
   </si>
   <si>
     <t>RES 470 OHM 1% 1/16W 0402</t>
@@ -265,7 +244,7 @@
     <t>RES SMD 10K OHM 0.1% 1/16W 0402</t>
   </si>
   <si>
-    <t>RES 2.2K OHM 1% 1/20W 0201</t>
+    <t>RES SMD 2.2K OHM 1% 1/16W 0402</t>
   </si>
   <si>
     <t>RES 100K OHM 1% 1/16W 0402</t>
@@ -298,9 +277,6 @@
     <t>Footprint</t>
   </si>
   <si>
-    <t>CAP-0201</t>
-  </si>
-  <si>
     <t>Cap-0402</t>
   </si>
   <si>
@@ -337,9 +313,6 @@
     <t>SOT-523_</t>
   </si>
   <si>
-    <t>Res-0201</t>
-  </si>
-  <si>
     <t>Res-0402</t>
   </si>
   <si>
@@ -373,10 +346,10 @@
     <t>Manufacturer Part Number</t>
   </si>
   <si>
-    <t>CC0201MRX5R6BB105</t>
-  </si>
-  <si>
-    <t>CC0201KRX5R6BB104</t>
+    <t>CC0402KRX5R7BB105, GRM155R61E105KA12D</t>
+  </si>
+  <si>
+    <t>GRM155R71C104KA88D</t>
   </si>
   <si>
     <t>CL05A475MO5NUNC</t>
@@ -385,15 +358,9 @@
     <t>CL05A106MP5NUNC</t>
   </si>
   <si>
-    <t>CC0402KRX5R7BB105, GRM155R61E105KA12D</t>
-  </si>
-  <si>
     <t>CC0402KRX5R6BB684</t>
   </si>
   <si>
-    <t>GRM155R71C104KA88D</t>
-  </si>
-  <si>
     <t>1N5819HW-7-F</t>
   </si>
   <si>
@@ -424,16 +391,13 @@
     <t>DMG1012T-7</t>
   </si>
   <si>
-    <t>RC0201FR-0710KL</t>
+    <t>RC0402FR-0710KL, RT0402BRD0710KL</t>
   </si>
   <si>
     <t>CRCW04021K00FKEDHP, RC0402FR-071KL</t>
   </si>
   <si>
-    <t>RC0201FR-074K7L</t>
-  </si>
-  <si>
-    <t>RC0402FR-0710KL, RT0402BRD0710KL</t>
+    <t>RC0402FR-074K7L</t>
   </si>
   <si>
     <t>RC0402FR-07470RL</t>
@@ -451,7 +415,7 @@
     <t>RT0402BRD0710KL</t>
   </si>
   <si>
-    <t>RC0201FR-072K2L</t>
+    <t>RC0402FR-072K2L</t>
   </si>
   <si>
     <t>RC0402FR-07100KL</t>
@@ -484,18 +448,18 @@
     <t>Manufacturer</t>
   </si>
   <si>
+    <t>Yageo, Murata</t>
+  </si>
+  <si>
+    <t>Murata</t>
+  </si>
+  <si>
+    <t>Samsung</t>
+  </si>
+  <si>
     <t>Yageo</t>
   </si>
   <si>
-    <t>Samsung</t>
-  </si>
-  <si>
-    <t>Yageo, Murata</t>
-  </si>
-  <si>
-    <t>Murata</t>
-  </si>
-  <si>
     <t>Diodes</t>
   </si>
   <si>
@@ -547,7 +511,7 @@
     <t>1uF</t>
   </si>
   <si>
-    <t>100nF</t>
+    <t>0.1uF</t>
   </si>
   <si>
     <t>4.7uF</t>
@@ -557,9 +521,6 @@
   </si>
   <si>
     <t>680nF</t>
-  </si>
-  <si>
-    <t>0.1uF</t>
   </si>
   <si>
     <t>4.7uH</t>
@@ -1094,7 +1055,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
@@ -1129,28 +1090,28 @@
         <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>173</v>
+        <v>161</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="11">
         <f>ROW(B3) - ROW($B$2)</f>
@@ -1160,56 +1121,56 @@
         <v>2</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>154</v>
+        <v>142</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>174</v>
+        <v>162</v>
       </c>
       <c r="J3" s="7">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="11">
-        <f t="shared" ref="B4:B38" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B36" si="0">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="13" t="s">
         <v>2</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>118</v>
+        <v>109</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>154</v>
+        <v>143</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="J4" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1218,26 +1179,26 @@
         <f>ROW(B5) - ROW($B$2)</f>
         <v>3</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="13" t="s">
         <v>2</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="J5" s="7">
         <v>2</v>
@@ -1253,53 +1214,53 @@
         <v>2</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>155</v>
+        <v>144</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>177</v>
+        <v>165</v>
       </c>
       <c r="J6" s="9">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="11">
         <f>ROW(B7) - ROW($B$2)</f>
         <v>5</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="J7" s="7">
         <v>2</v>
@@ -1312,28 +1273,28 @@
         <v>6</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>178</v>
+        <v>113</v>
       </c>
       <c r="J8" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1343,56 +1304,56 @@
         <v>7</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>179</v>
+        <v>114</v>
       </c>
       <c r="J9" s="7">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="11">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>4</v>
+        <v>180</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>124</v>
+        <v>88</v>
       </c>
       <c r="J10" s="9">
         <v>1</v>
@@ -1408,59 +1369,57 @@
         <v>4</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>159</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="H11" s="7"/>
       <c r="I11" s="8" t="s">
-        <v>125</v>
+        <v>89</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="11">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>193</v>
+        <v>5</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>160</v>
+        <v>143</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>96</v>
+        <v>167</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="11">
         <f>ROW(B13) - ROW($B$2)</f>
@@ -1470,20 +1429,22 @@
         <v>5</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="H13" s="7"/>
+        <v>91</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>149</v>
+      </c>
       <c r="I13" s="8" t="s">
-        <v>97</v>
+        <v>168</v>
       </c>
       <c r="J13" s="7">
         <v>1</v>
@@ -1499,25 +1460,25 @@
         <v>6</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>180</v>
+        <v>118</v>
       </c>
       <c r="J14" s="9">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1527,25 +1488,25 @@
         <v>13</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>99</v>
+        <v>119</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>181</v>
+        <v>119</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -1558,56 +1519,56 @@
         <v>14</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="J16" s="9">
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="11">
         <f>ROW(B17) - ROW($B$2)</f>
         <v>15</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="J17" s="7">
         <v>1</v>
@@ -1619,89 +1580,91 @@
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C18" s="13" t="s">
-        <v>9</v>
+      <c r="C18" s="12" t="s">
+        <v>7</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>164</v>
+        <v>146</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="J18" s="9">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="11">
         <f>ROW(B19) - ROW($B$2)</f>
         <v>17</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>165</v>
+        <v>145</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>132</v>
+        <v>169</v>
       </c>
       <c r="J19" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="11">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C20" s="13"/>
+      <c r="C20" s="13" t="s">
+        <v>9</v>
+      </c>
       <c r="D20" s="9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>133</v>
+        <v>170</v>
       </c>
       <c r="J20" s="9">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1711,93 +1674,93 @@
         <v>19</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="J21" s="7">
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="11">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>166</v>
+        <v>145</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
       <c r="J22" s="9">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="11">
         <f>ROW(B23) - ROW($B$2)</f>
         <v>21</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="J23" s="7">
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="11">
         <f t="shared" si="0"/>
@@ -1807,25 +1770,25 @@
         <v>10</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="J24" s="9">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1835,59 +1798,59 @@
         <v>23</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="J25" s="7">
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="11">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>167</v>
+        <v>145</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="J26" s="9">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1896,29 +1859,29 @@
         <f>ROW(B27) - ROW($B$2)</f>
         <v>25</v>
       </c>
-      <c r="C27" s="12" t="s">
-        <v>11</v>
+      <c r="C27" s="13" t="s">
+        <v>9</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="J27" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1928,124 +1891,124 @@
         <v>26</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="J28" s="9">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="11">
         <f>ROW(B29) - ROW($B$2)</f>
         <v>27</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>189</v>
+        <v>133</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="11">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>190</v>
+        <v>134</v>
       </c>
       <c r="J30" s="9">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="11">
         <f>ROW(B31) - ROW($B$2)</f>
         <v>29</v>
       </c>
       <c r="C31" s="12" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E31" s="8" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="H31" s="7" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="I31" s="8" t="s">
-        <v>191</v>
+        <v>135</v>
       </c>
       <c r="J31" s="7">
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="11">
         <f t="shared" si="0"/>
@@ -2055,84 +2018,84 @@
         <v>12</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="I32" s="10" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="J32" s="9">
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="11">
         <f>ROW(B33) - ROW($B$2)</f>
         <v>31</v>
       </c>
       <c r="C33" s="12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="I33" s="8" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="11">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C34" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F34" s="9" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="J34" s="9">
         <v>1</v>
@@ -2148,22 +2111,22 @@
         <v>13</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>171</v>
+        <v>147</v>
       </c>
       <c r="I35" s="8" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
@@ -2176,120 +2139,27 @@
         <v>34</v>
       </c>
       <c r="C36" s="13" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>172</v>
+        <v>159</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="J36" s="9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="1"/>
-      <c r="B37" s="11">
-        <f>ROW(B37) - ROW($B$2)</f>
-        <v>35</v>
-      </c>
-      <c r="C37" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D37" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="E37" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="F37" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="G37" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="H37" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="I37" s="8" t="s">
-        <v>150</v>
-      </c>
-      <c r="J37" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="1"/>
-      <c r="B38" s="11">
-        <f t="shared" si="0"/>
-        <v>36</v>
-      </c>
-      <c r="C38" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D38" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="E38" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="F38" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="G38" s="10" t="s">
-        <v>151</v>
-      </c>
-      <c r="H38" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="I38" s="10" t="s">
-        <v>151</v>
-      </c>
-      <c r="J38" s="9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="1"/>
-      <c r="B39" s="11">
-        <f>ROW(B39) - ROW($B$2)</f>
-        <v>37</v>
-      </c>
-      <c r="C39" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D39" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="E39" s="8" t="s">
-        <v>90</v>
-      </c>
-      <c r="F39" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="G39" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="H39" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="I39" s="8" t="s">
-        <v>152</v>
-      </c>
-      <c r="J39" s="7">
         <v>1</v>
       </c>
     </row>

</xml_diff>